<commit_message>
Add detailed logging for traffic data scraping process from Kemenhub Hubud
- Initialized scraping for domestic flight data from UPG airport covering the period from January 2020 to May 2026.
- Logged the total periods to be scraped and the number of previously scraped periods.
- Implemented CSRF token retrieval with retry logic and logging for each attempt.
- Added logs for each month processed, indicating success or skipping of already scraped data.
- Summarized the scraping results, including total requested periods, successful scrapes, and failures.
- Saved output in both CSV and Excel formats, with confirmation logs for successful file saves.
</commit_message>
<xml_diff>
--- a/lalinud_UPG_domestik_2020-01_2026-05.xlsx
+++ b/lalinud_UPG_domestik_2020-01_2026-05.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O37"/>
+  <dimension ref="A1:O78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2448,6 +2448,2179 @@
         <v>6154</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2023-01</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="n">
+        <v>3249</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>3249</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>387363</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>231570</v>
+      </c>
+      <c r="H38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="2" t="n">
+        <v>189440</v>
+      </c>
+      <c r="J38" s="2" t="n">
+        <v>3783656</v>
+      </c>
+      <c r="K38" s="2" t="n">
+        <v>2912100</v>
+      </c>
+      <c r="L38" s="2" t="n">
+        <v>3564054</v>
+      </c>
+      <c r="M38" s="2" t="n">
+        <v>4074465</v>
+      </c>
+      <c r="N38" s="2" t="n">
+        <v>106</v>
+      </c>
+      <c r="O38" s="2" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>2023-02</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>2938</v>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>2937</v>
+      </c>
+      <c r="F39" s="3" t="n">
+        <v>359565</v>
+      </c>
+      <c r="G39" s="3" t="n">
+        <v>200998</v>
+      </c>
+      <c r="H39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="3" t="n">
+        <v>179810</v>
+      </c>
+      <c r="J39" s="3" t="n">
+        <v>3574421</v>
+      </c>
+      <c r="K39" s="3" t="n">
+        <v>2939418</v>
+      </c>
+      <c r="L39" s="3" t="n">
+        <v>3155519</v>
+      </c>
+      <c r="M39" s="3" t="n">
+        <v>3438727</v>
+      </c>
+      <c r="N39" s="3" t="n">
+        <v>133</v>
+      </c>
+      <c r="O39" s="3" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2023-03</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="n">
+        <v>3159</v>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>3164</v>
+      </c>
+      <c r="F40" s="2" t="n">
+        <v>407505</v>
+      </c>
+      <c r="G40" s="2" t="n">
+        <v>226098</v>
+      </c>
+      <c r="H40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="2" t="n">
+        <v>197153</v>
+      </c>
+      <c r="J40" s="2" t="n">
+        <v>3844440</v>
+      </c>
+      <c r="K40" s="2" t="n">
+        <v>3375831</v>
+      </c>
+      <c r="L40" s="2" t="n">
+        <v>3571945</v>
+      </c>
+      <c r="M40" s="2" t="n">
+        <v>3811797</v>
+      </c>
+      <c r="N40" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="O40" s="2" t="n">
+        <v>2011</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>2023-04</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>3021</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>3022</v>
+      </c>
+      <c r="F41" s="3" t="n">
+        <v>403028</v>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>214056</v>
+      </c>
+      <c r="H41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="3" t="n">
+        <v>179390</v>
+      </c>
+      <c r="J41" s="3" t="n">
+        <v>3857692</v>
+      </c>
+      <c r="K41" s="3" t="n">
+        <v>2836292</v>
+      </c>
+      <c r="L41" s="3" t="n">
+        <v>3640510</v>
+      </c>
+      <c r="M41" s="3" t="n">
+        <v>3433438</v>
+      </c>
+      <c r="N41" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="O41" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2023-05</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="n">
+        <v>3749</v>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>3746</v>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>497964</v>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>292087</v>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="2" t="n">
+        <v>239553</v>
+      </c>
+      <c r="J42" s="2" t="n">
+        <v>4265893</v>
+      </c>
+      <c r="K42" s="2" t="n">
+        <v>3442745</v>
+      </c>
+      <c r="L42" s="2" t="n">
+        <v>4282222</v>
+      </c>
+      <c r="M42" s="2" t="n">
+        <v>4750967</v>
+      </c>
+      <c r="N42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O42" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>2023-06</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>3433</v>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>3427</v>
+      </c>
+      <c r="F43" s="3" t="n">
+        <v>442773</v>
+      </c>
+      <c r="G43" s="3" t="n">
+        <v>241544</v>
+      </c>
+      <c r="H43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="3" t="n">
+        <v>200771</v>
+      </c>
+      <c r="J43" s="3" t="n">
+        <v>3827614</v>
+      </c>
+      <c r="K43" s="3" t="n">
+        <v>3010306</v>
+      </c>
+      <c r="L43" s="3" t="n">
+        <v>3812918</v>
+      </c>
+      <c r="M43" s="3" t="n">
+        <v>3890283</v>
+      </c>
+      <c r="N43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O43" s="3" t="n">
+        <v>2387</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2023-07</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>3562</v>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>3556</v>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>469960</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>289998</v>
+      </c>
+      <c r="H44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="2" t="n">
+        <v>220755</v>
+      </c>
+      <c r="J44" s="2" t="n">
+        <v>3348117</v>
+      </c>
+      <c r="K44" s="2" t="n">
+        <v>2867202</v>
+      </c>
+      <c r="L44" s="2" t="n">
+        <v>4144357</v>
+      </c>
+      <c r="M44" s="2" t="n">
+        <v>4631101</v>
+      </c>
+      <c r="N44" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O44" s="2" t="n">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>2023-08</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>3183</v>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>3182</v>
+      </c>
+      <c r="F45" s="3" t="n">
+        <v>402204</v>
+      </c>
+      <c r="G45" s="3" t="n">
+        <v>224701</v>
+      </c>
+      <c r="H45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" s="3" t="n">
+        <v>192034</v>
+      </c>
+      <c r="J45" s="3" t="n">
+        <v>3466360</v>
+      </c>
+      <c r="K45" s="3" t="n">
+        <v>3649033</v>
+      </c>
+      <c r="L45" s="3" t="n">
+        <v>3466360</v>
+      </c>
+      <c r="M45" s="3" t="n">
+        <v>3647441</v>
+      </c>
+      <c r="N45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O45" s="3" t="n">
+        <v>1293</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>2023-09</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>3253</v>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>3251</v>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>411555</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>236372</v>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" s="2" t="n">
+        <v>183838</v>
+      </c>
+      <c r="J46" s="2" t="n">
+        <v>3581185</v>
+      </c>
+      <c r="K46" s="2" t="n">
+        <v>3039095</v>
+      </c>
+      <c r="L46" s="2" t="n">
+        <v>3629482</v>
+      </c>
+      <c r="M46" s="2" t="n">
+        <v>3646771</v>
+      </c>
+      <c r="N46" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O46" s="2" t="n">
+        <v>1089</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>2023-10</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>2484</v>
+      </c>
+      <c r="E47" s="3" t="n">
+        <v>2520</v>
+      </c>
+      <c r="F47" s="3" t="n">
+        <v>335259</v>
+      </c>
+      <c r="G47" s="3" t="n">
+        <v>184050</v>
+      </c>
+      <c r="H47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" s="3" t="n">
+        <v>2330627</v>
+      </c>
+      <c r="K47" s="3" t="n">
+        <v>1832638</v>
+      </c>
+      <c r="L47" s="3" t="n">
+        <v>2800895</v>
+      </c>
+      <c r="M47" s="3" t="n">
+        <v>1637223</v>
+      </c>
+      <c r="N47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O47" s="3" t="n">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>2023-11</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="n">
+        <v>2778</v>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>2797</v>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>400403</v>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>412180</v>
+      </c>
+      <c r="H48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" s="2" t="n">
+        <v>2898619</v>
+      </c>
+      <c r="K48" s="2" t="n">
+        <v>2318076</v>
+      </c>
+      <c r="L48" s="2" t="n">
+        <v>3283521</v>
+      </c>
+      <c r="M48" s="2" t="n">
+        <v>1832223</v>
+      </c>
+      <c r="N48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O48" s="2" t="n">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>2023-12</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>1656</v>
+      </c>
+      <c r="E49" s="3" t="n">
+        <v>1648</v>
+      </c>
+      <c r="F49" s="3" t="n">
+        <v>241821</v>
+      </c>
+      <c r="G49" s="3" t="n">
+        <v>237005</v>
+      </c>
+      <c r="H49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="3" t="n">
+        <v>3935</v>
+      </c>
+      <c r="J49" s="3" t="n">
+        <v>2026615</v>
+      </c>
+      <c r="K49" s="3" t="n">
+        <v>1528043</v>
+      </c>
+      <c r="L49" s="3" t="n">
+        <v>2016549</v>
+      </c>
+      <c r="M49" s="3" t="n">
+        <v>1098910</v>
+      </c>
+      <c r="N49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O49" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2024-01</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="n">
+        <v>2290</v>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>2279</v>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>291764</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>310902</v>
+      </c>
+      <c r="H50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="2" t="n">
+        <v>127465</v>
+      </c>
+      <c r="J50" s="2" t="n">
+        <v>2890863</v>
+      </c>
+      <c r="K50" s="2" t="n">
+        <v>2358952</v>
+      </c>
+      <c r="L50" s="2" t="n">
+        <v>2591239</v>
+      </c>
+      <c r="M50" s="2" t="n">
+        <v>1821704</v>
+      </c>
+      <c r="N50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O50" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>2024-02</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>2205</v>
+      </c>
+      <c r="E51" s="3" t="n">
+        <v>2211</v>
+      </c>
+      <c r="F51" s="3" t="n">
+        <v>301331</v>
+      </c>
+      <c r="G51" s="3" t="n">
+        <v>313756</v>
+      </c>
+      <c r="H51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" s="3" t="n">
+        <v>124153</v>
+      </c>
+      <c r="J51" s="3" t="n">
+        <v>3246646</v>
+      </c>
+      <c r="K51" s="3" t="n">
+        <v>2852943</v>
+      </c>
+      <c r="L51" s="3" t="n">
+        <v>2594109</v>
+      </c>
+      <c r="M51" s="3" t="n">
+        <v>1692110</v>
+      </c>
+      <c r="N51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O51" s="3" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="n">
+        <v>2383</v>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>2380</v>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>334130</v>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>335213</v>
+      </c>
+      <c r="H52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" s="2" t="n">
+        <v>145552</v>
+      </c>
+      <c r="J52" s="2" t="n">
+        <v>3857231</v>
+      </c>
+      <c r="K52" s="2" t="n">
+        <v>2955846</v>
+      </c>
+      <c r="L52" s="2" t="n">
+        <v>2997818</v>
+      </c>
+      <c r="M52" s="2" t="n">
+        <v>1983218</v>
+      </c>
+      <c r="N52" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O52" s="2" t="n">
+        <v>2759</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>2024-04</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>2776</v>
+      </c>
+      <c r="E53" s="3" t="n">
+        <v>2760</v>
+      </c>
+      <c r="F53" s="3" t="n">
+        <v>412240</v>
+      </c>
+      <c r="G53" s="3" t="n">
+        <v>409790</v>
+      </c>
+      <c r="H53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" s="3" t="n">
+        <v>80782</v>
+      </c>
+      <c r="J53" s="3" t="n">
+        <v>3403247</v>
+      </c>
+      <c r="K53" s="3" t="n">
+        <v>2511897</v>
+      </c>
+      <c r="L53" s="3" t="n">
+        <v>3807604</v>
+      </c>
+      <c r="M53" s="3" t="n">
+        <v>2559641</v>
+      </c>
+      <c r="N53" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="O53" s="3" t="n">
+        <v>1930</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>2024-05</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="n">
+        <v>2645</v>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>2637</v>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>363457</v>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>378739</v>
+      </c>
+      <c r="H54" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="2" t="n">
+        <v>154659</v>
+      </c>
+      <c r="J54" s="2" t="n">
+        <v>3541918</v>
+      </c>
+      <c r="K54" s="2" t="n">
+        <v>2729246</v>
+      </c>
+      <c r="L54" s="2" t="n">
+        <v>3100665</v>
+      </c>
+      <c r="M54" s="2" t="n">
+        <v>2030945</v>
+      </c>
+      <c r="N54" s="2" t="n">
+        <v>1993</v>
+      </c>
+      <c r="O54" s="2" t="n">
+        <v>2505</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>2024-06</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>2688</v>
+      </c>
+      <c r="E55" s="3" t="n">
+        <v>2694</v>
+      </c>
+      <c r="F55" s="3" t="n">
+        <v>392895</v>
+      </c>
+      <c r="G55" s="3" t="n">
+        <v>378681</v>
+      </c>
+      <c r="H55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="3" t="n">
+        <v>153289</v>
+      </c>
+      <c r="J55" s="3" t="n">
+        <v>3537272</v>
+      </c>
+      <c r="K55" s="3" t="n">
+        <v>2452298</v>
+      </c>
+      <c r="L55" s="3" t="n">
+        <v>3414905</v>
+      </c>
+      <c r="M55" s="3" t="n">
+        <v>2159879</v>
+      </c>
+      <c r="N55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" s="3" t="n">
+        <v>1733</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2024-07</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="n">
+        <v>2784</v>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>2783</v>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>396910</v>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>418660</v>
+      </c>
+      <c r="H56" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="2" t="n">
+        <v>104816</v>
+      </c>
+      <c r="J56" s="2" t="n">
+        <v>3503496</v>
+      </c>
+      <c r="K56" s="2" t="n">
+        <v>2563335</v>
+      </c>
+      <c r="L56" s="2" t="n">
+        <v>3484647</v>
+      </c>
+      <c r="M56" s="2" t="n">
+        <v>2483001</v>
+      </c>
+      <c r="N56" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O56" s="2" t="n">
+        <v>1602</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>2668</v>
+      </c>
+      <c r="E57" s="3" t="n">
+        <v>2659</v>
+      </c>
+      <c r="F57" s="3" t="n">
+        <v>377395</v>
+      </c>
+      <c r="G57" s="3" t="n">
+        <v>383498</v>
+      </c>
+      <c r="H57" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" s="3" t="n">
+        <v>156996</v>
+      </c>
+      <c r="J57" s="3" t="n">
+        <v>3587643</v>
+      </c>
+      <c r="K57" s="3" t="n">
+        <v>2730030</v>
+      </c>
+      <c r="L57" s="3" t="n">
+        <v>3202464</v>
+      </c>
+      <c r="M57" s="3" t="n">
+        <v>2135685</v>
+      </c>
+      <c r="N57" s="3" t="n">
+        <v>4805</v>
+      </c>
+      <c r="O57" s="3" t="n">
+        <v>2036</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2024-09</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="n">
+        <v>2654</v>
+      </c>
+      <c r="E58" s="2" t="n">
+        <v>2638</v>
+      </c>
+      <c r="F58" s="2" t="n">
+        <v>369846</v>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>379846</v>
+      </c>
+      <c r="H58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" s="2" t="n">
+        <v>156081</v>
+      </c>
+      <c r="J58" s="2" t="n">
+        <v>3472767</v>
+      </c>
+      <c r="K58" s="2" t="n">
+        <v>2761911</v>
+      </c>
+      <c r="L58" s="2" t="n">
+        <v>3113636</v>
+      </c>
+      <c r="M58" s="2" t="n">
+        <v>1990221</v>
+      </c>
+      <c r="N58" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O58" s="2" t="n">
+        <v>1984</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>2024-10</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>2658</v>
+      </c>
+      <c r="E59" s="3" t="n">
+        <v>2642</v>
+      </c>
+      <c r="F59" s="3" t="n">
+        <v>374140</v>
+      </c>
+      <c r="G59" s="3" t="n">
+        <v>378225</v>
+      </c>
+      <c r="H59" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" s="3" t="n">
+        <v>159884</v>
+      </c>
+      <c r="J59" s="3" t="n">
+        <v>3738547</v>
+      </c>
+      <c r="K59" s="3" t="n">
+        <v>2845765</v>
+      </c>
+      <c r="L59" s="3" t="n">
+        <v>3130815</v>
+      </c>
+      <c r="M59" s="3" t="n">
+        <v>1991052</v>
+      </c>
+      <c r="N59" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O59" s="3" t="n">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="n">
+        <v>2664</v>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>2657</v>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>352972</v>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>356060</v>
+      </c>
+      <c r="H60" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" s="2" t="n">
+        <v>147562</v>
+      </c>
+      <c r="J60" s="2" t="n">
+        <v>3916143</v>
+      </c>
+      <c r="K60" s="2" t="n">
+        <v>2850962</v>
+      </c>
+      <c r="L60" s="2" t="n">
+        <v>2956180</v>
+      </c>
+      <c r="M60" s="2" t="n">
+        <v>2042285</v>
+      </c>
+      <c r="N60" s="2" t="n">
+        <v>1308</v>
+      </c>
+      <c r="O60" s="2" t="n">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>2931</v>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>2910</v>
+      </c>
+      <c r="F61" s="3" t="n">
+        <v>414784</v>
+      </c>
+      <c r="G61" s="3" t="n">
+        <v>387117</v>
+      </c>
+      <c r="H61" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" s="3" t="n">
+        <v>156410</v>
+      </c>
+      <c r="J61" s="3" t="n">
+        <v>4069203</v>
+      </c>
+      <c r="K61" s="3" t="n">
+        <v>2936894</v>
+      </c>
+      <c r="L61" s="3" t="n">
+        <v>3581230</v>
+      </c>
+      <c r="M61" s="3" t="n">
+        <v>2202759</v>
+      </c>
+      <c r="N61" s="3" t="n">
+        <v>5088</v>
+      </c>
+      <c r="O61" s="3" t="n">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="n">
+        <v>2611</v>
+      </c>
+      <c r="E62" s="2" t="n">
+        <v>2611</v>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>354143</v>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>377017</v>
+      </c>
+      <c r="H62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" s="2" t="n">
+        <v>129159</v>
+      </c>
+      <c r="J62" s="2" t="n">
+        <v>3627966</v>
+      </c>
+      <c r="K62" s="2" t="n">
+        <v>3091946</v>
+      </c>
+      <c r="L62" s="2" t="n">
+        <v>3177653</v>
+      </c>
+      <c r="M62" s="2" t="n">
+        <v>2401384</v>
+      </c>
+      <c r="N62" s="2" t="n">
+        <v>130</v>
+      </c>
+      <c r="O62" s="2" t="n">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>2297</v>
+      </c>
+      <c r="E63" s="3" t="n">
+        <v>2301</v>
+      </c>
+      <c r="F63" s="3" t="n">
+        <v>322045</v>
+      </c>
+      <c r="G63" s="3" t="n">
+        <v>330499</v>
+      </c>
+      <c r="H63" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" s="3" t="n">
+        <v>119336</v>
+      </c>
+      <c r="J63" s="3" t="n">
+        <v>3159692</v>
+      </c>
+      <c r="K63" s="3" t="n">
+        <v>2449517</v>
+      </c>
+      <c r="L63" s="3" t="n">
+        <v>2853893</v>
+      </c>
+      <c r="M63" s="3" t="n">
+        <v>1910662</v>
+      </c>
+      <c r="N63" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O63" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="n">
+        <v>2282</v>
+      </c>
+      <c r="E64" s="2" t="n">
+        <v>2279</v>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>326149</v>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>299275</v>
+      </c>
+      <c r="H64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I64" s="2" t="n">
+        <v>115828</v>
+      </c>
+      <c r="J64" s="2" t="n">
+        <v>3689172</v>
+      </c>
+      <c r="K64" s="2" t="n">
+        <v>2806859</v>
+      </c>
+      <c r="L64" s="2" t="n">
+        <v>2993453</v>
+      </c>
+      <c r="M64" s="2" t="n">
+        <v>1748947</v>
+      </c>
+      <c r="N64" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="O64" s="2" t="n">
+        <v>1636</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>2802</v>
+      </c>
+      <c r="E65" s="3" t="n">
+        <v>2811</v>
+      </c>
+      <c r="F65" s="3" t="n">
+        <v>379166</v>
+      </c>
+      <c r="G65" s="3" t="n">
+        <v>409247</v>
+      </c>
+      <c r="H65" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I65" s="3" t="n">
+        <v>134292</v>
+      </c>
+      <c r="J65" s="3" t="n">
+        <v>3312096</v>
+      </c>
+      <c r="K65" s="3" t="n">
+        <v>2655316</v>
+      </c>
+      <c r="L65" s="3" t="n">
+        <v>3425164</v>
+      </c>
+      <c r="M65" s="3" t="n">
+        <v>2707026</v>
+      </c>
+      <c r="N65" s="3" t="n">
+        <v>74</v>
+      </c>
+      <c r="O65" s="3" t="n">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="n">
+        <v>2446</v>
+      </c>
+      <c r="E66" s="2" t="n">
+        <v>2442</v>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>324682</v>
+      </c>
+      <c r="G66" s="2" t="n">
+        <v>324055</v>
+      </c>
+      <c r="H66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" s="2" t="n">
+        <v>120280</v>
+      </c>
+      <c r="J66" s="2" t="n">
+        <v>3698328</v>
+      </c>
+      <c r="K66" s="2" t="n">
+        <v>3154181</v>
+      </c>
+      <c r="L66" s="2" t="n">
+        <v>2699678</v>
+      </c>
+      <c r="M66" s="2" t="n">
+        <v>1862998</v>
+      </c>
+      <c r="N66" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O66" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>2699</v>
+      </c>
+      <c r="E67" s="3" t="n">
+        <v>2697</v>
+      </c>
+      <c r="F67" s="3" t="n">
+        <v>380199</v>
+      </c>
+      <c r="G67" s="3" t="n">
+        <v>378266</v>
+      </c>
+      <c r="H67" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" s="3" t="n">
+        <v>138260</v>
+      </c>
+      <c r="J67" s="3" t="n">
+        <v>3872686</v>
+      </c>
+      <c r="K67" s="3" t="n">
+        <v>3353486</v>
+      </c>
+      <c r="L67" s="3" t="n">
+        <v>3257815</v>
+      </c>
+      <c r="M67" s="3" t="n">
+        <v>2164821</v>
+      </c>
+      <c r="N67" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O67" s="3" t="n">
+        <v>2418</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>3056</v>
+      </c>
+      <c r="E68" s="2" t="n">
+        <v>3057</v>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>403176</v>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>422019</v>
+      </c>
+      <c r="H68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" s="2" t="n">
+        <v>155329</v>
+      </c>
+      <c r="J68" s="2" t="n">
+        <v>3571769</v>
+      </c>
+      <c r="K68" s="2" t="n">
+        <v>3593131</v>
+      </c>
+      <c r="L68" s="2" t="n">
+        <v>3419028</v>
+      </c>
+      <c r="M68" s="2" t="n">
+        <v>3665018</v>
+      </c>
+      <c r="N68" s="2" t="n">
+        <v>138</v>
+      </c>
+      <c r="O68" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>2841</v>
+      </c>
+      <c r="E69" s="3" t="n">
+        <v>2834</v>
+      </c>
+      <c r="F69" s="3" t="n">
+        <v>375542</v>
+      </c>
+      <c r="G69" s="3" t="n">
+        <v>379557</v>
+      </c>
+      <c r="H69" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" s="3" t="n">
+        <v>140654</v>
+      </c>
+      <c r="J69" s="3" t="n">
+        <v>3208715</v>
+      </c>
+      <c r="K69" s="3" t="n">
+        <v>2984419</v>
+      </c>
+      <c r="L69" s="3" t="n">
+        <v>2946871</v>
+      </c>
+      <c r="M69" s="3" t="n">
+        <v>3204054</v>
+      </c>
+      <c r="N69" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O69" s="3" t="n">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>2665</v>
+      </c>
+      <c r="E70" s="2" t="n">
+        <v>2650</v>
+      </c>
+      <c r="F70" s="2" t="n">
+        <v>358102</v>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>363313</v>
+      </c>
+      <c r="H70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" s="2" t="n">
+        <v>134311</v>
+      </c>
+      <c r="J70" s="2" t="n">
+        <v>2928833</v>
+      </c>
+      <c r="K70" s="2" t="n">
+        <v>2852608</v>
+      </c>
+      <c r="L70" s="2" t="n">
+        <v>2772910</v>
+      </c>
+      <c r="M70" s="2" t="n">
+        <v>2989663</v>
+      </c>
+      <c r="N70" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="O70" s="2" t="n">
+        <v>1231</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>3007</v>
+      </c>
+      <c r="E71" s="3" t="n">
+        <v>2994</v>
+      </c>
+      <c r="F71" s="3" t="n">
+        <v>407914</v>
+      </c>
+      <c r="G71" s="3" t="n">
+        <v>415614</v>
+      </c>
+      <c r="H71" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I71" s="3" t="n">
+        <v>164583</v>
+      </c>
+      <c r="J71" s="3" t="n">
+        <v>3458131</v>
+      </c>
+      <c r="K71" s="3" t="n">
+        <v>3389760</v>
+      </c>
+      <c r="L71" s="3" t="n">
+        <v>3136751</v>
+      </c>
+      <c r="M71" s="3" t="n">
+        <v>3564744</v>
+      </c>
+      <c r="N71" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O71" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="n">
+        <v>2976</v>
+      </c>
+      <c r="E72" s="2" t="n">
+        <v>2977</v>
+      </c>
+      <c r="F72" s="2" t="n">
+        <v>407765</v>
+      </c>
+      <c r="G72" s="2" t="n">
+        <v>412871</v>
+      </c>
+      <c r="H72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I72" s="2" t="n">
+        <v>166565</v>
+      </c>
+      <c r="J72" s="2" t="n">
+        <v>3540841</v>
+      </c>
+      <c r="K72" s="2" t="n">
+        <v>3358929</v>
+      </c>
+      <c r="L72" s="2" t="n">
+        <v>3195288</v>
+      </c>
+      <c r="M72" s="2" t="n">
+        <v>3518987</v>
+      </c>
+      <c r="N72" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O72" s="2" t="n">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>3090</v>
+      </c>
+      <c r="E73" s="3" t="n">
+        <v>3091</v>
+      </c>
+      <c r="F73" s="3" t="n">
+        <v>432685</v>
+      </c>
+      <c r="G73" s="3" t="n">
+        <v>409294</v>
+      </c>
+      <c r="H73" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I73" s="3" t="n">
+        <v>168725</v>
+      </c>
+      <c r="J73" s="3" t="n">
+        <v>3710901</v>
+      </c>
+      <c r="K73" s="3" t="n">
+        <v>3807225</v>
+      </c>
+      <c r="L73" s="3" t="n">
+        <v>3473673</v>
+      </c>
+      <c r="M73" s="3" t="n">
+        <v>2803956</v>
+      </c>
+      <c r="N73" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="O73" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>2726</v>
+      </c>
+      <c r="E74" s="2" t="n">
+        <v>2723</v>
+      </c>
+      <c r="F74" s="2" t="n">
+        <v>332206</v>
+      </c>
+      <c r="G74" s="2" t="n">
+        <v>358703</v>
+      </c>
+      <c r="H74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I74" s="2" t="n">
+        <v>133965</v>
+      </c>
+      <c r="J74" s="2" t="n">
+        <v>2896603</v>
+      </c>
+      <c r="K74" s="2" t="n">
+        <v>3013593</v>
+      </c>
+      <c r="L74" s="2" t="n">
+        <v>2734221</v>
+      </c>
+      <c r="M74" s="2" t="n">
+        <v>1997543</v>
+      </c>
+      <c r="N74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O74" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E75" s="3" t="n">
+        <v>1171</v>
+      </c>
+      <c r="F75" s="3" t="n">
+        <v>120591</v>
+      </c>
+      <c r="G75" s="3" t="n">
+        <v>127733</v>
+      </c>
+      <c r="H75" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I75" s="3" t="n">
+        <v>49443</v>
+      </c>
+      <c r="J75" s="3" t="n">
+        <v>1274481</v>
+      </c>
+      <c r="K75" s="3" t="n">
+        <v>1412778</v>
+      </c>
+      <c r="L75" s="3" t="n">
+        <v>1004538</v>
+      </c>
+      <c r="M75" s="3" t="n">
+        <v>702645</v>
+      </c>
+      <c r="N75" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O75" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>3104</v>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>3118</v>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>409630</v>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>398415</v>
+      </c>
+      <c r="H76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I76" s="2" t="n">
+        <v>152109</v>
+      </c>
+      <c r="J76" s="2" t="n">
+        <v>2807052</v>
+      </c>
+      <c r="K76" s="2" t="n">
+        <v>3297336</v>
+      </c>
+      <c r="L76" s="2" t="n">
+        <v>3515247</v>
+      </c>
+      <c r="M76" s="2" t="n">
+        <v>3569445</v>
+      </c>
+      <c r="N76" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="O76" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>2827</v>
+      </c>
+      <c r="E77" s="3" t="n">
+        <v>2834</v>
+      </c>
+      <c r="F77" s="3" t="n">
+        <v>297976</v>
+      </c>
+      <c r="G77" s="3" t="n">
+        <v>321424</v>
+      </c>
+      <c r="H77" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I77" s="3" t="n">
+        <v>131597</v>
+      </c>
+      <c r="J77" s="3" t="n">
+        <v>2558925</v>
+      </c>
+      <c r="K77" s="3" t="n">
+        <v>2816687</v>
+      </c>
+      <c r="L77" s="3" t="n">
+        <v>2385188</v>
+      </c>
+      <c r="M77" s="3" t="n">
+        <v>2857755</v>
+      </c>
+      <c r="N77" s="3" t="n">
+        <v>102</v>
+      </c>
+      <c r="O77" s="3" t="n">
+        <v>6226</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>UPG</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Domestik</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>1724</v>
+      </c>
+      <c r="E78" s="2" t="n">
+        <v>1723</v>
+      </c>
+      <c r="F78" s="2" t="n">
+        <v>73536</v>
+      </c>
+      <c r="G78" s="2" t="n">
+        <v>72465</v>
+      </c>
+      <c r="H78" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I78" s="2" t="n">
+        <v>26348</v>
+      </c>
+      <c r="J78" s="2" t="n">
+        <v>866128</v>
+      </c>
+      <c r="K78" s="2" t="n">
+        <v>993581</v>
+      </c>
+      <c r="L78" s="2" t="n">
+        <v>560972</v>
+      </c>
+      <c r="M78" s="2" t="n">
+        <v>624985</v>
+      </c>
+      <c r="N78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O78" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>